<commit_message>
url finder and connector completed
</commit_message>
<xml_diff>
--- a/contacts.xlsx
+++ b/contacts.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70BAFDC6-16DD-45D5-B14D-1B26B1ED51E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="39">
   <si>
     <t>Full Name</t>
   </si>
@@ -44,53 +43,115 @@
     <t>Notes</t>
   </si>
   <si>
+    <t>Sahil Shaikh</t>
+  </si>
+  <si>
     <t>Dextero Business Solutions</t>
   </si>
   <si>
-    <t>https://in.linkedin.com/in/akash-bansode</t>
+    <t>https://in.linkedin.com/in/sahil-shaikh-4a4a941b6</t>
   </si>
   <si>
     <t>URL Found</t>
   </si>
   <si>
+    <t>1/7/2026</t>
+  </si>
+  <si>
+    <t>Sent</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Sahil Shaikh</t>
+    <t>Found via Google</t>
+  </si>
+  <si>
+    <t>Shrutika Shinde</t>
   </si>
   <si>
     <t xml:space="preserve">ITM Group of Institutions </t>
   </si>
   <si>
-    <t>Shrutika Shinde</t>
+    <t>https://www.linkedin.com/in/shrutika-shinde-10287a3a0</t>
+  </si>
+  <si>
+    <t>Found via LinkedIn</t>
   </si>
   <si>
     <t>Mitali Araj</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/mitali180401araj</t>
+  </si>
+  <si>
     <t>Mrudula Rehenge</t>
   </si>
   <si>
+    <t>https://in.linkedin.com/in/akash-koli-aa716918</t>
+  </si>
+  <si>
     <t>Akash Gupta</t>
   </si>
   <si>
     <t>Lokmanya Tilak college  of Engineering</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/aakash-gupta-15807a239</t>
+  </si>
+  <si>
     <t>Yashika Sharma</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/yashika-sharma04</t>
+  </si>
+  <si>
+    <t>Bhavik Sapat</t>
+  </si>
+  <si>
+    <t>Dextero Business Solution Pvt.Ltd.</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/bhaviksapat</t>
+  </si>
+  <si>
+    <t>Sachin Gupta</t>
+  </si>
+  <si>
+    <t>Vivekanand Education Society's Polytechnic</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/sachin-gupta-a008633a3</t>
+  </si>
+  <si>
+    <t>Sanjay Shetty</t>
+  </si>
+  <si>
+    <t>Dextero</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/sanjay-shetty-100b657</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <color theme="10"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -113,8 +174,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -130,6 +195,34 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="Table1" displayName="Table1" ref="A1:I10" totalsRowShown="1" headerRowCount="0">
+  <autoFilter>
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
+    <filterColumn colId="7" hiddenButton="1"/>
+    <filterColumn colId="8" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="9">
+    <tableColumn id="1" name="Full Name"/>
+    <tableColumn id="2" name="Company"/>
+    <tableColumn id="3" name="LinkedIn URL"/>
+    <tableColumn id="4" name="URL Status"/>
+    <tableColumn id="5" name="Connection Sent Date"/>
+    <tableColumn id="6" name="Connection Status"/>
+    <tableColumn id="7" name="Message Sent Date"/>
+    <tableColumn id="8" name="Message Text"/>
+    <tableColumn id="9" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -453,18 +546,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="37.90625" customWidth="1"/>
-    <col min="2" max="2" width="33.26953125" customWidth="1"/>
-    <col min="3" max="3" width="41.453125" customWidth="1"/>
+    <col min="2" max="2" width="43.54296875" customWidth="1"/>
+    <col min="3" max="3" width="53.26953125" customWidth="1"/>
     <col min="4" max="4" width="18.7265625" customWidth="1"/>
     <col min="5" max="5" width="22.36328125" customWidth="1"/>
+    <col min="6" max="6" width="36.81640625" customWidth="1"/>
+    <col min="7" max="7" width="18.7265625" customWidth="1"/>
+    <col min="8" max="8" width="14.1796875" customWidth="1"/>
+    <col min="9" max="9" width="18.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -493,77 +590,224 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
         <v>12</v>
       </c>
-      <c r="H2" t="s">
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" t="s">
         <v>12</v>
       </c>
-      <c r="I2" t="s">
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="I7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" ht="14.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="I8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" ht="14.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="I9" t="s">
         <v>20</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="10" ht="14.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" t="s">
         <v>14</v>
+      </c>
+      <c r="I10" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>